<commit_message>
Update projections: qb_2026_combined.xlsx, rb_2026_combined.xlsx, wr_2026_combined.xlsx, te_2026_combined.xlsx, kicker_2026_combined.xlsx, def_2026_combined.xlsx
</commit_message>
<xml_diff>
--- a/projections/def_2026_combined.xlsx
+++ b/projections/def_2026_combined.xlsx
@@ -7265,7 +7265,7 @@
         <v>0.1796</v>
       </c>
       <c r="I118" t="n">
-        <v>23.89</v>
+        <v>23.98</v>
       </c>
       <c r="J118" t="n">
         <v>349</v>
@@ -11270,7 +11270,7 @@
         <v>0.201</v>
       </c>
       <c r="I207" t="n">
-        <v>19.47</v>
+        <v>19.53</v>
       </c>
       <c r="J207" t="n">
         <v>294.6</v>
@@ -12440,7 +12440,7 @@
         <v>0.1649</v>
       </c>
       <c r="I233" t="n">
-        <v>19.35</v>
+        <v>19.58</v>
       </c>
       <c r="J233" t="n">
         <v>303.7</v>
@@ -12452,7 +12452,7 @@
         <v>-2.074</v>
       </c>
       <c r="M233" t="n">
-        <v>24.583</v>
+        <v>22.621</v>
       </c>
     </row>
     <row r="234">
@@ -15500,7 +15500,7 @@
         <v>0.1281</v>
       </c>
       <c r="I301" t="n">
-        <v>20.75</v>
+        <v>20.61</v>
       </c>
       <c r="J301" t="n">
         <v>291.1</v>
@@ -18560,7 +18560,7 @@
         <v>0.1375</v>
       </c>
       <c r="I369" t="n">
-        <v>21.71</v>
+        <v>21.54</v>
       </c>
       <c r="J369" t="n">
         <v>309.5</v>

</xml_diff>